<commit_message>
feat(lia): agent Goals, rectification expert et parcours locataire
Architecture Lia réactive (SharedState, intake, agent), Pro Briefing et
rectification expert (charge, cas sensibles, prise en charge). Références
légales, flags qualification, multi-réclamations et évolutions Flutter locataire.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Processus application.xlsx
+++ b/Processus application.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ewald\Desktop\LE LOCATAIRE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{43999528-67CD-42C7-833B-76206230F1E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECB7F578-4FE8-4088-80F1-113DB0605314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{C4DB092D-13B6-4916-9EAC-D3601856AEC5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{C4DB092D-13B6-4916-9EAC-D3601856AEC5}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="121">
   <si>
     <t>Processus application LE LOCATAIRE</t>
   </si>
@@ -258,15 +258,221 @@
   <si>
     <t>gestion des prestataires pour travaux locatif</t>
   </si>
+  <si>
+    <t>une réclamation</t>
+  </si>
+  <si>
+    <t>fuite sous évier</t>
+  </si>
+  <si>
+    <t>questiion 1</t>
+  </si>
+  <si>
+    <t>depuis quand avez-vous constater la fuite</t>
+  </si>
+  <si>
+    <t>réponse probales</t>
+  </si>
+  <si>
+    <t>question 2</t>
+  </si>
+  <si>
+    <t>réponse probable</t>
+  </si>
+  <si>
+    <t>question 3</t>
+  </si>
+  <si>
+    <t>(quoi?)</t>
+  </si>
+  <si>
+    <t>(quand?)</t>
+  </si>
+  <si>
+    <t>avez-vous fait quelque chose nettoyer le siphond, mis du produit pour déboucher?</t>
+  </si>
+  <si>
+    <t>oui j'en ais mis hier</t>
+  </si>
+  <si>
+    <t>l'eau de votre lavabo s'écoule normalement?</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>réponse probale</t>
+  </si>
+  <si>
+    <t>oui elle s'écoule normalement</t>
+  </si>
+  <si>
+    <t>pré-diagnostic</t>
+  </si>
+  <si>
+    <t>depuis mon entrée dans le logement</t>
+  </si>
+  <si>
+    <t>oui</t>
+  </si>
+  <si>
+    <t>non</t>
+  </si>
+  <si>
+    <t>nettoyer le siphon, metter des produits vendu dans le marché et revenez ver nous</t>
+  </si>
+  <si>
+    <t>depuis mon entrée dans le logement (si dans les 4 mois et moins de 6 mois)</t>
+  </si>
+  <si>
+    <t>locataire entrant passage de l'entrepris qui à fait la REL ou d'un plombier</t>
+  </si>
+  <si>
+    <t>1 er cas</t>
+  </si>
+  <si>
+    <t>2 eme cas</t>
+  </si>
+  <si>
+    <t>fuite de toiture</t>
+  </si>
+  <si>
+    <t>penser à vous protéger vos effet personnels</t>
+  </si>
+  <si>
+    <t>oui, daccord</t>
+  </si>
+  <si>
+    <t>3eme cas</t>
+  </si>
+  <si>
+    <t>pas d'électricité dans la chambre</t>
+  </si>
+  <si>
+    <t>depuis quand</t>
+  </si>
+  <si>
+    <t>avez-vous tous débranchés et relevé le disjoncteur</t>
+  </si>
+  <si>
+    <t>le disjonteur ne reste pas</t>
+  </si>
+  <si>
+    <t>faite le, débrancher tous et faite monter le disjoncteur</t>
+  </si>
+  <si>
+    <t>il reste enclanché</t>
+  </si>
+  <si>
+    <t>probablement un appareil defectueux</t>
+  </si>
+  <si>
+    <t>oui, mais dès que jutilise un appareil le compteur saute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">êtes vous à jour de votre abonnement, avez-vous eu un retard de payement </t>
+  </si>
+  <si>
+    <t>oui à jour et pas de retard ce mois ci</t>
+  </si>
+  <si>
+    <t>oui à jour je viens de payer ma facture j'étais en retard</t>
+  </si>
+  <si>
+    <t>cela doit être un problème électrique</t>
+  </si>
+  <si>
+    <t>avez-vous appeler votre fournissuer d'électricité</t>
+  </si>
+  <si>
+    <t>quand il pleut</t>
+  </si>
+  <si>
+    <t>Comptes de test (démo)</t>
+  </si>
+  <si>
+    <t>Profil</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Mot de passe</t>
+  </si>
+  <si>
+    <t>Page après login</t>
+  </si>
+  <si>
+    <t>Référent V1</t>
+  </si>
+  <si>
+    <t>demo.referent@lelocataire.test</t>
+  </si>
+  <si>
+    <t>DemoReferent1!</t>
+  </si>
+  <si>
+    <t>/agent/reclamations</t>
+  </si>
+  <si>
+    <t>demo.bailleur@lelocataire.test</t>
+  </si>
+  <si>
+    <t>DemoBailleur1!</t>
+  </si>
+  <si>
+    <t>/bailleur/dashboard</t>
+  </si>
+  <si>
+    <t>Locataire</t>
+  </si>
+  <si>
+    <t>demo.locataire@lelocataire.test</t>
+  </si>
+  <si>
+    <t>DemoLocataire1!</t>
+  </si>
+  <si>
+    <t>App mobile</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -280,7 +486,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -604,11 +810,162 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -636,18 +993,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -661,24 +1006,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -686,15 +1013,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -733,6 +1051,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -742,8 +1066,97 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2672,23 +3085,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="17"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
@@ -2758,20 +3171,20 @@
       <c r="P6" s="8"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="21" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="8"/>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="27"/>
-      <c r="K7" s="28"/>
+      <c r="E7" s="53"/>
+      <c r="F7" s="53"/>
+      <c r="G7" s="53"/>
+      <c r="H7" s="53"/>
+      <c r="I7" s="53"/>
+      <c r="J7" s="53"/>
+      <c r="K7" s="54"/>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
@@ -2797,17 +3210,17 @@
     </row>
     <row r="9" spans="2:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C9" s="8"/>
-      <c r="D9" s="35" t="s">
+      <c r="D9" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="37"/>
-      <c r="F9" s="36"/>
+      <c r="E9" s="51"/>
+      <c r="F9" s="40"/>
       <c r="G9" s="8"/>
-      <c r="H9" s="35" t="s">
+      <c r="H9" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="I9" s="36"/>
-      <c r="L9" s="32" t="s">
+      <c r="I9" s="40"/>
+      <c r="L9" s="22" t="s">
         <v>40</v>
       </c>
       <c r="M9" s="8"/>
@@ -2820,17 +3233,17 @@
         <v>35</v>
       </c>
       <c r="C10" s="8"/>
-      <c r="D10" s="29" t="s">
+      <c r="D10" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="30"/>
-      <c r="F10" s="31"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="50"/>
       <c r="G10" s="8"/>
-      <c r="H10" s="33" t="s">
+      <c r="H10" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="I10" s="34"/>
-      <c r="L10" s="32" t="s">
+      <c r="I10" s="24"/>
+      <c r="L10" s="22" t="s">
         <v>12</v>
       </c>
       <c r="M10" s="8"/>
@@ -2839,7 +3252,7 @@
       <c r="P10" s="8"/>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B11" s="24"/>
+      <c r="B11" s="20"/>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
       <c r="E11" s="8"/>
@@ -2856,7 +3269,7 @@
       <c r="P11" s="8"/>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B12" s="24"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
@@ -2873,7 +3286,7 @@
       <c r="P12" s="8"/>
     </row>
     <row r="13" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="24"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
@@ -2890,140 +3303,140 @@
       <c r="P13" s="8"/>
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B14" s="38"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39" t="s">
+      <c r="B14" s="25"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="39"/>
-      <c r="F14" s="40"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="27"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
-      <c r="J14" s="46"/>
-      <c r="K14" s="39"/>
-      <c r="L14" s="39" t="s">
+      <c r="J14" s="33"/>
+      <c r="K14" s="26"/>
+      <c r="L14" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="M14" s="39"/>
-      <c r="N14" s="40"/>
+      <c r="M14" s="26"/>
+      <c r="N14" s="27"/>
       <c r="O14" s="8"/>
       <c r="P14" s="8"/>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B15" s="41" t="s">
+      <c r="B15" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="43" t="s">
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="30" t="s">
         <v>12</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8"/>
-      <c r="J15" s="47" t="s">
+      <c r="J15" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="K15" s="42"/>
-      <c r="L15" s="42"/>
-      <c r="M15" s="42"/>
-      <c r="N15" s="43" t="s">
+      <c r="K15" s="29"/>
+      <c r="L15" s="29"/>
+      <c r="M15" s="29"/>
+      <c r="N15" s="30" t="s">
         <v>11</v>
       </c>
       <c r="O15" s="8"/>
       <c r="P15" s="8"/>
     </row>
     <row r="16" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="44"/>
-      <c r="C16" s="45"/>
-      <c r="D16" s="45" t="s">
+      <c r="B16" s="31"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="E16" s="45"/>
-      <c r="F16" s="34"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="24"/>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
-      <c r="J16" s="48"/>
-      <c r="K16" s="45"/>
-      <c r="L16" s="45" t="s">
+      <c r="J16" s="35"/>
+      <c r="K16" s="32"/>
+      <c r="L16" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="M16" s="45"/>
-      <c r="N16" s="34"/>
+      <c r="M16" s="32"/>
+      <c r="N16" s="24"/>
       <c r="O16" s="8"/>
       <c r="P16" s="8"/>
     </row>
     <row r="17" spans="2:31" x14ac:dyDescent="0.25">
       <c r="B17" s="5"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="42"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
-      <c r="J17" s="42"/>
-      <c r="K17" s="42"/>
-      <c r="L17" s="42"/>
-      <c r="M17" s="42"/>
-      <c r="N17" s="42"/>
+      <c r="J17" s="29"/>
+      <c r="K17" s="29"/>
+      <c r="L17" s="29"/>
+      <c r="M17" s="29"/>
+      <c r="N17" s="29"/>
       <c r="O17" s="8"/>
       <c r="P17" s="8"/>
     </row>
     <row r="18" spans="2:31" x14ac:dyDescent="0.25">
       <c r="B18" s="5"/>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="42"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="42"/>
-      <c r="K18" s="42"/>
-      <c r="L18" s="42"/>
-      <c r="M18" s="42"/>
-      <c r="N18" s="42"/>
+      <c r="J18" s="29"/>
+      <c r="K18" s="29"/>
+      <c r="L18" s="29"/>
+      <c r="M18" s="29"/>
+      <c r="N18" s="29"/>
       <c r="O18" s="8"/>
       <c r="P18" s="8"/>
     </row>
     <row r="19" spans="2:31" x14ac:dyDescent="0.25">
       <c r="B19" s="5"/>
-      <c r="C19" s="42"/>
-      <c r="D19" s="42"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="42"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
-      <c r="J19" s="42"/>
-      <c r="K19" s="42"/>
-      <c r="L19" s="42"/>
-      <c r="M19" s="42"/>
-      <c r="N19" s="42"/>
+      <c r="J19" s="29"/>
+      <c r="K19" s="29"/>
+      <c r="L19" s="29"/>
+      <c r="M19" s="29"/>
+      <c r="N19" s="29"/>
       <c r="O19" s="8"/>
       <c r="P19" s="8"/>
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.25">
       <c r="I20" s="8"/>
-      <c r="J20" s="42"/>
-      <c r="K20" s="42"/>
-      <c r="L20" s="42"/>
-      <c r="M20" s="42"/>
-      <c r="N20" s="42"/>
+      <c r="J20" s="29"/>
+      <c r="K20" s="29"/>
+      <c r="L20" s="29"/>
+      <c r="M20" s="29"/>
+      <c r="N20" s="29"/>
       <c r="O20" s="8"/>
       <c r="P20" s="8"/>
     </row>
     <row r="21" spans="2:31" x14ac:dyDescent="0.25">
       <c r="I21" s="8"/>
-      <c r="J21" s="42"/>
-      <c r="K21" s="42"/>
-      <c r="L21" s="42"/>
-      <c r="M21" s="42"/>
-      <c r="N21" s="42"/>
+      <c r="J21" s="29"/>
+      <c r="K21" s="29"/>
+      <c r="L21" s="29"/>
+      <c r="M21" s="29"/>
+      <c r="N21" s="29"/>
       <c r="O21" s="8"/>
       <c r="P21" s="8"/>
       <c r="X21" s="1" t="s">
@@ -3032,22 +3445,22 @@
     </row>
     <row r="22" spans="2:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="5"/>
-      <c r="C22" s="42"/>
-      <c r="D22" s="42" t="s">
+      <c r="C22" s="29"/>
+      <c r="D22" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
       <c r="G22" s="8"/>
       <c r="H22" s="8" t="s">
         <v>12</v>
       </c>
       <c r="I22" s="8"/>
-      <c r="J22" s="42"/>
-      <c r="K22" s="42"/>
-      <c r="L22" s="42"/>
-      <c r="M22" s="42"/>
-      <c r="N22" s="42"/>
+      <c r="J22" s="29"/>
+      <c r="K22" s="29"/>
+      <c r="L22" s="29"/>
+      <c r="M22" s="29"/>
+      <c r="N22" s="29"/>
       <c r="O22" s="8"/>
       <c r="P22" s="8"/>
     </row>
@@ -3055,27 +3468,27 @@
       <c r="B23" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="42"/>
+      <c r="C23" s="29"/>
       <c r="D23" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="E23" s="42"/>
-      <c r="F23" s="32" t="s">
+      <c r="E23" s="29"/>
+      <c r="F23" s="22" t="s">
         <v>44</v>
       </c>
       <c r="G23" s="8"/>
-      <c r="H23" s="32" t="s">
+      <c r="H23" s="22" t="s">
         <v>46</v>
       </c>
       <c r="I23" s="8"/>
-      <c r="J23" s="32" t="s">
+      <c r="J23" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="K23" s="42"/>
-      <c r="L23" s="32" t="s">
+      <c r="K23" s="29"/>
+      <c r="L23" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="M23" s="42"/>
+      <c r="M23" s="29"/>
       <c r="N23" s="3" t="s">
         <v>52</v>
       </c>
@@ -3090,9 +3503,9 @@
     </row>
     <row r="24" spans="2:31" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I24" s="8"/>
-      <c r="K24" s="42"/>
-      <c r="M24" s="42"/>
-      <c r="N24" s="42"/>
+      <c r="K24" s="29"/>
+      <c r="M24" s="29"/>
+      <c r="N24" s="29"/>
       <c r="O24" s="8"/>
       <c r="P24" s="1" t="s">
         <v>54</v>
@@ -3100,10 +3513,10 @@
     </row>
     <row r="25" spans="2:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I25" s="8"/>
-      <c r="J25" s="42"/>
-      <c r="K25" s="42"/>
-      <c r="L25" s="42"/>
-      <c r="M25" s="42"/>
+      <c r="J25" s="29"/>
+      <c r="K25" s="29"/>
+      <c r="L25" s="29"/>
+      <c r="M25" s="29"/>
       <c r="O25" s="8"/>
       <c r="P25" s="8"/>
       <c r="Q25" s="8">
@@ -3118,34 +3531,34 @@
     </row>
     <row r="26" spans="2:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="5"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="42"/>
-      <c r="F26" s="42"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
       <c r="I26" s="8"/>
-      <c r="J26" s="42"/>
-      <c r="K26" s="42"/>
-      <c r="L26" s="42"/>
-      <c r="M26" s="42"/>
-      <c r="N26" s="42"/>
+      <c r="J26" s="29"/>
+      <c r="K26" s="29"/>
+      <c r="L26" s="29"/>
+      <c r="M26" s="29"/>
+      <c r="N26" s="29"/>
       <c r="O26" s="8"/>
       <c r="P26" s="8"/>
       <c r="Q26" s="8"/>
       <c r="W26" s="1">
         <v>1</v>
       </c>
-      <c r="X26" s="49" t="s">
+      <c r="X26" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="Y26" s="50"/>
-      <c r="Z26" s="51"/>
-      <c r="AB26" s="35" t="s">
+      <c r="Y26" s="37"/>
+      <c r="Z26" s="38"/>
+      <c r="AB26" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="AC26" s="36"/>
-      <c r="AE26" s="52" t="s">
+      <c r="AC26" s="40"/>
+      <c r="AE26" s="41" t="s">
         <v>61</v>
       </c>
     </row>
@@ -3159,19 +3572,19 @@
       <c r="T27" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="AE27" s="53"/>
+      <c r="AE27" s="42"/>
     </row>
     <row r="28" spans="2:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="Q28" s="8"/>
       <c r="W28" s="1">
         <v>0</v>
       </c>
-      <c r="X28" s="49" t="s">
+      <c r="X28" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="Y28" s="50"/>
-      <c r="Z28" s="51"/>
-      <c r="AE28" s="53"/>
+      <c r="Y28" s="37"/>
+      <c r="Z28" s="38"/>
+      <c r="AE28" s="42"/>
     </row>
     <row r="29" spans="2:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="Q29" s="8">
@@ -3183,7 +3596,7 @@
       <c r="T29" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="AE29" s="54"/>
+      <c r="AE29" s="43"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B36" s="9"/>
@@ -3192,11 +3605,11 @@
       <c r="E36" s="10"/>
       <c r="F36" s="10"/>
       <c r="G36" s="10"/>
-      <c r="H36" s="21" t="s">
+      <c r="H36" s="17" t="s">
         <v>21</v>
       </c>
       <c r="I36" s="10"/>
-      <c r="J36" s="21" t="s">
+      <c r="J36" s="17" t="s">
         <v>21</v>
       </c>
       <c r="K36" s="10"/>
@@ -3204,7 +3617,7 @@
         <v>11</v>
       </c>
       <c r="M36" s="10"/>
-      <c r="N36" s="21" t="s">
+      <c r="N36" s="17" t="s">
         <v>21</v>
       </c>
       <c r="O36" s="10"/>
@@ -3216,7 +3629,7 @@
         <v>12</v>
       </c>
       <c r="S36" s="10"/>
-      <c r="T36" s="21" t="s">
+      <c r="T36" s="17" t="s">
         <v>21</v>
       </c>
       <c r="U36" s="10"/>
@@ -3300,7 +3713,7 @@
         <v>11</v>
       </c>
       <c r="E39" s="6"/>
-      <c r="F39" s="22" t="s">
+      <c r="F39" s="18" t="s">
         <v>21</v>
       </c>
       <c r="G39" s="6"/>
@@ -3350,7 +3763,7 @@
       <c r="Y40" s="13"/>
     </row>
     <row r="41" spans="2:25" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="23" t="s">
+      <c r="B41" s="19" t="s">
         <v>1</v>
       </c>
       <c r="C41" s="6"/>
@@ -3388,13 +3801,13 @@
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
-      <c r="H42" s="22" t="s">
+      <c r="H42" s="18" t="s">
         <v>21</v>
       </c>
       <c r="I42" s="6"/>
       <c r="J42" s="6"/>
       <c r="K42" s="5"/>
-      <c r="L42" s="22" t="s">
+      <c r="L42" s="18" t="s">
         <v>21</v>
       </c>
       <c r="M42" s="6"/>
@@ -3402,7 +3815,7 @@
         <v>11</v>
       </c>
       <c r="O42" s="6"/>
-      <c r="P42" s="22" t="s">
+      <c r="P42" s="18" t="s">
         <v>21</v>
       </c>
       <c r="Q42" s="6"/>
@@ -3510,11 +3923,11 @@
       <c r="Y45" s="16"/>
     </row>
     <row r="46" spans="2:25" x14ac:dyDescent="0.25">
-      <c r="F46" s="17" t="s">
+      <c r="F46" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="G46" s="17"/>
-      <c r="H46" s="17"/>
+      <c r="G46" s="44"/>
+      <c r="H46" s="44"/>
       <c r="L46" s="1" t="s">
         <v>21</v>
       </c>
@@ -3527,11 +3940,11 @@
       <c r="D48" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F48" s="18" t="s">
+      <c r="F48" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="G48" s="19"/>
-      <c r="H48" s="20"/>
+      <c r="G48" s="46"/>
+      <c r="H48" s="47"/>
       <c r="I48" s="7"/>
       <c r="J48" s="7"/>
       <c r="L48" s="3" t="s">
@@ -3727,4 +4140,462 @@
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F8B93DC-E733-41E3-A5BD-BBBCB27C9391}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B7:M39"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="36.85546875" customWidth="1"/>
+    <col min="5" max="5" width="36" style="55" customWidth="1"/>
+    <col min="6" max="6" width="43" style="55" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" style="55" customWidth="1"/>
+    <col min="8" max="8" width="18.5703125" style="55" customWidth="1"/>
+    <col min="9" max="9" width="18.28515625" style="55" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="12" max="12" width="21" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="7" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="55" t="s">
+        <v>64</v>
+      </c>
+      <c r="F7" s="55" t="s">
+        <v>66</v>
+      </c>
+      <c r="G7" s="55" t="s">
+        <v>67</v>
+      </c>
+      <c r="H7" s="55" t="s">
+        <v>68</v>
+      </c>
+      <c r="I7" s="55" t="s">
+        <v>69</v>
+      </c>
+      <c r="J7" s="55" t="s">
+        <v>76</v>
+      </c>
+      <c r="K7" s="55"/>
+      <c r="L7" s="55" t="s">
+        <v>78</v>
+      </c>
+      <c r="M7" s="55"/>
+    </row>
+    <row r="8" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E8" s="56" t="s">
+        <v>71</v>
+      </c>
+      <c r="G8" s="56" t="s">
+        <v>70</v>
+      </c>
+      <c r="I8" s="55" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+      <c r="B9" s="59" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="60" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="60"/>
+      <c r="E9" s="61" t="s">
+        <v>65</v>
+      </c>
+      <c r="F9" s="61" t="s">
+        <v>65</v>
+      </c>
+      <c r="G9" s="61" t="s">
+        <v>72</v>
+      </c>
+      <c r="H9" s="61" t="s">
+        <v>73</v>
+      </c>
+      <c r="I9" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="J9" s="61" t="s">
+        <v>77</v>
+      </c>
+      <c r="K9" s="61"/>
+      <c r="L9" s="61"/>
+      <c r="M9" s="62"/>
+    </row>
+    <row r="10" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+      <c r="B10" s="63"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="58"/>
+      <c r="F10" s="58"/>
+      <c r="G10" s="58" t="s">
+        <v>72</v>
+      </c>
+      <c r="H10" s="58" t="s">
+        <v>81</v>
+      </c>
+      <c r="I10" s="58" t="s">
+        <v>74</v>
+      </c>
+      <c r="J10" s="58" t="s">
+        <v>77</v>
+      </c>
+      <c r="K10" s="58"/>
+      <c r="L10" s="58" t="s">
+        <v>82</v>
+      </c>
+      <c r="M10" s="64"/>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B11" s="63"/>
+      <c r="C11" s="57"/>
+      <c r="D11" s="57"/>
+      <c r="E11" s="58"/>
+      <c r="F11" s="58"/>
+      <c r="G11" s="58"/>
+      <c r="H11" s="58"/>
+      <c r="I11" s="58"/>
+      <c r="J11" s="57"/>
+      <c r="K11" s="57"/>
+      <c r="L11" s="57"/>
+      <c r="M11" s="64"/>
+    </row>
+    <row r="12" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+      <c r="B12" s="63"/>
+      <c r="C12" s="57"/>
+      <c r="D12" s="57"/>
+      <c r="E12" s="58"/>
+      <c r="F12" s="58" t="s">
+        <v>83</v>
+      </c>
+      <c r="G12" s="58" t="s">
+        <v>72</v>
+      </c>
+      <c r="H12" s="58" t="s">
+        <v>81</v>
+      </c>
+      <c r="I12" s="58" t="s">
+        <v>74</v>
+      </c>
+      <c r="J12" s="58" t="s">
+        <v>80</v>
+      </c>
+      <c r="K12" s="58"/>
+      <c r="L12" s="58" t="s">
+        <v>84</v>
+      </c>
+      <c r="M12" s="64"/>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B13" s="63"/>
+      <c r="C13" s="57"/>
+      <c r="D13" s="57"/>
+      <c r="E13" s="58"/>
+      <c r="F13" s="58"/>
+      <c r="G13" s="58"/>
+      <c r="H13" s="58"/>
+      <c r="I13" s="58"/>
+      <c r="J13" s="57"/>
+      <c r="K13" s="57"/>
+      <c r="L13" s="57"/>
+      <c r="M13" s="64"/>
+    </row>
+    <row r="14" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+      <c r="B14" s="63"/>
+      <c r="C14" s="57"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="58"/>
+      <c r="F14" s="58"/>
+      <c r="G14" s="58" t="s">
+        <v>72</v>
+      </c>
+      <c r="H14" s="58" t="s">
+        <v>80</v>
+      </c>
+      <c r="I14" s="58" t="s">
+        <v>74</v>
+      </c>
+      <c r="J14" s="58" t="s">
+        <v>81</v>
+      </c>
+      <c r="K14" s="58"/>
+      <c r="L14" s="58" t="s">
+        <v>12</v>
+      </c>
+      <c r="M14" s="64"/>
+    </row>
+    <row r="15" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="65"/>
+      <c r="C15" s="66"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="67"/>
+      <c r="F15" s="67"/>
+      <c r="G15" s="67"/>
+      <c r="H15" s="67"/>
+      <c r="I15" s="67"/>
+      <c r="J15" s="66"/>
+      <c r="K15" s="66"/>
+      <c r="L15" s="66"/>
+      <c r="M15" s="68"/>
+    </row>
+    <row r="18" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="2:13" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="69" t="s">
+        <v>86</v>
+      </c>
+      <c r="C19" s="70" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="70"/>
+      <c r="E19" s="71" t="s">
+        <v>65</v>
+      </c>
+      <c r="F19" s="71" t="s">
+        <v>104</v>
+      </c>
+      <c r="G19" s="71" t="s">
+        <v>88</v>
+      </c>
+      <c r="H19" s="71" t="s">
+        <v>89</v>
+      </c>
+      <c r="I19" s="71"/>
+      <c r="J19" s="70"/>
+      <c r="K19" s="70"/>
+      <c r="L19" s="71" t="s">
+        <v>12</v>
+      </c>
+      <c r="M19" s="72"/>
+    </row>
+    <row r="22" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="23" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="B23" s="59" t="s">
+        <v>90</v>
+      </c>
+      <c r="C23" s="61" t="s">
+        <v>91</v>
+      </c>
+      <c r="D23" s="60"/>
+      <c r="E23" s="61" t="s">
+        <v>92</v>
+      </c>
+      <c r="F23" s="61" t="s">
+        <v>79</v>
+      </c>
+      <c r="G23" s="61" t="s">
+        <v>93</v>
+      </c>
+      <c r="H23" s="61" t="s">
+        <v>80</v>
+      </c>
+      <c r="I23" s="61"/>
+      <c r="J23" s="61" t="s">
+        <v>94</v>
+      </c>
+      <c r="K23" s="61"/>
+      <c r="L23" s="60"/>
+      <c r="M23" s="73"/>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B24" s="63"/>
+      <c r="C24" s="57"/>
+      <c r="D24" s="57"/>
+      <c r="E24" s="58"/>
+      <c r="F24" s="58"/>
+      <c r="G24" s="58"/>
+      <c r="H24" s="58"/>
+      <c r="I24" s="58"/>
+      <c r="J24" s="57"/>
+      <c r="K24" s="57"/>
+      <c r="L24" s="57"/>
+      <c r="M24" s="64"/>
+    </row>
+    <row r="25" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+      <c r="B25" s="63"/>
+      <c r="C25" s="57"/>
+      <c r="D25" s="57"/>
+      <c r="E25" s="58"/>
+      <c r="F25" s="58"/>
+      <c r="G25" s="58"/>
+      <c r="H25" s="58" t="s">
+        <v>81</v>
+      </c>
+      <c r="I25" s="58" t="s">
+        <v>95</v>
+      </c>
+      <c r="J25" s="58" t="s">
+        <v>96</v>
+      </c>
+      <c r="K25" s="58" t="s">
+        <v>97</v>
+      </c>
+      <c r="L25" s="57"/>
+      <c r="M25" s="64"/>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B26" s="63"/>
+      <c r="C26" s="57"/>
+      <c r="D26" s="57"/>
+      <c r="E26" s="58"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="58"/>
+      <c r="H26" s="58"/>
+      <c r="I26" s="58"/>
+      <c r="J26" s="57"/>
+      <c r="K26" s="57"/>
+      <c r="L26" s="57"/>
+      <c r="M26" s="64"/>
+    </row>
+    <row r="27" spans="2:13" ht="75" x14ac:dyDescent="0.25">
+      <c r="B27" s="63"/>
+      <c r="C27" s="57"/>
+      <c r="D27" s="57"/>
+      <c r="E27" s="58"/>
+      <c r="F27" s="58"/>
+      <c r="G27" s="58"/>
+      <c r="H27" s="58" t="s">
+        <v>98</v>
+      </c>
+      <c r="I27" s="58" t="s">
+        <v>99</v>
+      </c>
+      <c r="J27" s="58" t="s">
+        <v>100</v>
+      </c>
+      <c r="K27" s="58" t="s">
+        <v>102</v>
+      </c>
+      <c r="L27" s="57"/>
+      <c r="M27" s="64"/>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B28" s="63"/>
+      <c r="C28" s="57"/>
+      <c r="D28" s="57"/>
+      <c r="E28" s="58"/>
+      <c r="F28" s="58"/>
+      <c r="G28" s="58"/>
+      <c r="H28" s="58"/>
+      <c r="I28" s="58"/>
+      <c r="J28" s="58"/>
+      <c r="K28" s="57"/>
+      <c r="L28" s="57"/>
+      <c r="M28" s="64"/>
+    </row>
+    <row r="29" spans="2:13" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="65"/>
+      <c r="C29" s="66"/>
+      <c r="D29" s="66"/>
+      <c r="E29" s="67"/>
+      <c r="F29" s="67"/>
+      <c r="G29" s="67"/>
+      <c r="H29" s="67"/>
+      <c r="I29" s="67"/>
+      <c r="J29" s="67" t="s">
+        <v>101</v>
+      </c>
+      <c r="K29" s="67" t="s">
+        <v>103</v>
+      </c>
+      <c r="L29" s="66"/>
+      <c r="M29" s="68"/>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="J30" s="55"/>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="J31" s="55"/>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="J32" s="55"/>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J33" s="55"/>
+    </row>
+    <row r="34" spans="2:10" ht="81" x14ac:dyDescent="0.3">
+      <c r="B34" s="74" t="s">
+        <v>105</v>
+      </c>
+      <c r="C34" s="75"/>
+      <c r="D34" s="75"/>
+      <c r="E34" s="75"/>
+      <c r="J34" s="55"/>
+    </row>
+    <row r="35" spans="2:10" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="B35" s="76"/>
+      <c r="C35" s="75"/>
+      <c r="D35" s="75"/>
+      <c r="E35" s="75"/>
+      <c r="J35" s="55"/>
+    </row>
+    <row r="36" spans="2:10" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="B36" s="77" t="s">
+        <v>106</v>
+      </c>
+      <c r="C36" s="77" t="s">
+        <v>107</v>
+      </c>
+      <c r="E36" s="77" t="s">
+        <v>108</v>
+      </c>
+      <c r="F36" s="77" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="B37" s="78" t="s">
+        <v>110</v>
+      </c>
+      <c r="C37" s="81" t="s">
+        <v>111</v>
+      </c>
+      <c r="E37" s="79" t="s">
+        <v>112</v>
+      </c>
+      <c r="F37" s="79" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="B38" s="78" t="s">
+        <v>23</v>
+      </c>
+      <c r="C38" s="79" t="s">
+        <v>114</v>
+      </c>
+      <c r="E38" s="79" t="s">
+        <v>115</v>
+      </c>
+      <c r="F38" s="79" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="39" spans="2:10" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="B39" s="78" t="s">
+        <v>117</v>
+      </c>
+      <c r="C39" s="79" t="s">
+        <v>118</v>
+      </c>
+      <c r="E39" s="79" t="s">
+        <v>119</v>
+      </c>
+      <c r="F39" s="80" t="s">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C37" r:id="rId1" xr:uid="{6ABF34E7-3C7F-424D-88B4-503ED3F4D7BE}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="43" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>